<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-03 La prune violette du marché
Réécriture vocale example4 : éclat de cageot, lunettes vécues.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-03.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La prune de la tarte</t>
+          <t>La prune violette du marché</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>boulangerie puis marché</t>
+          <t>marché : toiles, caisse de prunes, filet de coton, pain, balance, banc, pommes, menthe, œufs</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Mila, maman</t>
+          <t>Nino, Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut une prune bien ronde pour la tarte de maman. Il prend une molle. Mila, avec ses lunettes, voit une prune ferme au fond. Ils la portent dans le filet.</t>
+          <t>Une toile claque. Sur la caisse, un éclat de cageot brille. Nino veut une prune violette, maintenant, avec Mila. Il saisit trop vite : la prune tombe, le filet se coince. Sourire parti. Mila arrive, lunettes neuves. Un rire commence. Il ferme la bouche, tend une prune. Merci vécu. Il lève trop haut : le jus tache, les lunettes bougent. Il refuse de foncer. L'éclat de cageot tient. La prune est partagée.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le four du boulanger souffle une odeur de mie. Un peu de farine blanchit la planche. Le pain chaud croustille dans le sac. Une miette tombe près de la caisse. Maman tient un filet de coton. Le filet sent encore la lessive. Le sol est un peu collant. Tu as senti le pain, Nino ? Il est chaud. Oui. Il ira avec la tarte. Nino touche le sac de pain. Le papier est tiède. En ce moment, Nino regarde les prunes. Elles sont violettes et lisses. Une caisse sent le sucré. J'en veux une ronde. Pour la tarte. On en cherche une ferme. Pas trop molle. Mila arrive près de la caisse. Ses chaussures collent un peu au sol. Mila a des lunettes neuves. Mila a les cheveux lisses. Elle porte un gilet vert. Mila, tu cherches avec Nino. Tu m'aides, Mila ? Oui. Nino prend une prune. Elle cède un peu sous le doigt. Elle est molle. On la repose. Tout doux, dans la caisse. Mila se penche sur la caisse. Elle regarde au fond. Au fond. Celle-là.</t>
+          <t>Une toile claque au-dessus des prunes. J'entends la toile, maman ! Tu l'entends, au-dessus ? Oui, elle claque. Ça sent le sucré, un peu chaud. Tu le sens, Nino ? Oui, papa. Un cageot de bois est ouvert. Des prunes violettes y brillent. Sur la caisse, un éclat de cageot brille. Il brille, papa ! Tu le vois, sur le bois ? Oui, un petit point. Le filet de coton est prêt. Il gratte un peu. On le remplit, Nino ? Oui, avec une prune. Le pain chaud tape le bras de Nino. Il est tiède. Le papier croustille ? Oui, papa. À côté, des pommes rouges attendent. Elles sont lisses, maman. On verra les pommes après ? Après la prune. Une balance fait tic, tout près. J'entends le tic. C'est la balance ? Oui. En ce moment, Nino veut une prune. Je veux une prune, maintenant ! Une prune violette, maman. Avec Mila, Nino ? Oui, maman. Nino saisit trop vite une prune. La prune glisse entre ses doigts. Elle tombe dans le cageot. Elle est tombée ! Nino tire le filet trop vite. Le filet se coince au bord. Il est coincé ! Le coton, Nino ? Il tient au bois. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux la prune avec Mila ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Mila arrive près du cageot. Mila ! Ses chaussures collent un peu au sol. Mila a des lunettes neuves. Tu vois Mila, Nino ? Oui, papa. Elles brillent un peu. Elle porte un gilet vert. Tu viens, Mila ? Oui. Nino ouvre la bouche. Un petit rire commence. Oh. Nino ferme la bouche. Il regarde la caisse. Il tend une prune. Pour toi. Mila ne dit rien, d'abord. Elle compte les prunes des yeux. Celle-là. L'éclat de cageot tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le four du boulanger souffle une odeur de mie. Un peu de farine blanchit la planche. Le pain chaud croustille dans le sac. Une miette tombe près de la caisse. Maman tient un filet de coton. Le filet sent encore la lessive. Le sol est un peu collant. Tu as senti le pain, Nino ? Il est chaud. Oui. Il ira avec la tarte. Nino touche le sac de pain. Le papier est tiède. En ce moment, Nino regarde les prunes. Elles sont violettes et lisses. Une caisse sent le sucré. J'en veux une ronde. Pour la tarte. On en cherche une ferme. Pas trop molle. Mila arrive près de la caisse. Ses chaussures collent un peu au sol. Mila a des lunettes neuves. Mila a les cheveux lisses. Elle porte un gilet vert. Mila, tu cherches avec Nino. Tu m'aides, Mila ? Oui. Nino prend une prune. Elle cède un peu sous le doigt. Elle est molle. On la repose. Tout doux, dans la caisse. Mila se penche sur la caisse. Elle regarde au fond. Au fond. Celle-là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une toile claque au-dessus des prunes. J'entends la toile, maman ! Tu l'entends, au-dessus ? Oui, elle claque. Ça sent le sucré, un peu chaud. Tu le sens, Nino ? Oui, papa. Un cageot de bois est ouvert. Des prunes violettes y brillent. Sur la caisse, un &lt;emphasis level="moderate"&gt;éclat de cageot&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, sur le bois ? Oui, un petit point. Le filet de coton est prêt. Il gratte un peu. On le remplit, Nino ? Oui, avec une prune. Le pain chaud tape le bras de Nino. Il est tiède. Le papier croustille ? Oui, papa. À côté, des pommes rouges attendent. Elles sont lisses, maman. On verra les pommes après ? Après la prune. Une balance fait tic, tout près. J'entends le tic. C'est la balance ? Oui. En ce moment, Nino veut une prune. Je veux une prune, maintenant ! Une prune violette, maman. Avec Mila, Nino ? Oui, maman. Nino saisit trop vite une prune. La prune glisse entre ses doigts. Elle tombe dans le cageot. Elle est tombée ! Nino tire le filet trop vite. Le filet se coince au bord. Il est coincé ! Le coton, Nino ? Il tient au bois. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux la prune avec Mila ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Mila arrive près du cageot. Mila ! Ses chaussures collent un peu au sol. Mila a des lunettes neuves. Tu vois Mila, Nino ? Oui, papa. Elles brillent un peu. Elle porte un gilet vert. Tu viens, Mila ? Oui. Nino ouvre la bouche. Un petit rire commence. Oh. Nino ferme la bouche. Il regarde la caisse. Il tend une prune. Pour toi. Mila ne dit rien, d'abord. Elle compte les prunes des yeux. Celle-là. L'éclat de cageot tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maya est au marché avec maman. Inès arrive avec des lunettes neuves. Elles brillent un peu. Un camarade ouvre la bouche. Maya ne rit &lt;emphasis&gt;pas&lt;/emphasis&gt;. Il ne faut pas rire de l'apparence. Maman dit : on joue. On ne rit pas des lunettes, des cheveux ou d'un habit. Maya tend une prune à Inès. Elles marchent ensemble. Maya dit : tes lunettes sont là. C'est tout. Pas rire de l'apparence. [pause]</t>
+          <t>Une toile claque au-dessus des prunes. J'entends la toile, maman ! Tu l'entends, au-dessus ? Oui, elle claque. Ça sent le sucré, un peu chaud. Tu le sens, Nino ? Oui, papa. Un cageot de bois est ouvert. Des prunes violettes y brillent. Sur la caisse, un &lt;emphasis&gt;éclat de cageot&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, sur le bois ? Oui, un petit point. Le filet de coton est prêt. Il gratte un peu. On le remplit, Nino ? Oui, avec une prune. Le pain chaud tape le bras de Nino. Il est tiède. Le papier croustille ? Oui, papa. À côté, des pommes rouges attendent. Elles sont lisses, maman. On verra les pommes après ? Après la prune. Une balance fait tic, tout près. J'entends le tic. C'est la balance ? Oui. En ce moment, Nino veut une prune. Je veux une prune, maintenant ! Une prune violette, maman. Avec Mila, Nino ? Oui, maman. Nino saisit trop vite une prune. La prune glisse entre ses doigts. Elle tombe dans le cageot. Elle est tombée ! Nino tire le filet trop vite. Le filet se coince au bord. Il est coincé ! Le coton, Nino ? Il tient au bois. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux la prune avec Mila ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Mila arrive près du cageot. Mila ! Ses chaussures collent un peu au sol. Mila a des lunettes neuves. Tu vois Mila, Nino ? Oui, papa. Elles brillent un peu. Elle porte un gilet vert. Tu viens, Mila ? Oui. Nino ouvre la bouche. Un petit rire commence. Oh. Nino ferme la bouche. Il regarde la caisse. Il tend une prune. Pour toi. Mila ne dit rien, d'abord. Elle compte les prunes des yeux. Celle-là. L'éclat de cageot tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de cageot</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,46 +1321,85 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_prune_violette_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le four du boulanger souffle une odeur de mie.
-narrateur|Un peu de farine blanchit la planche.
-narrateur|Le pain chaud croustille dans le sac.
-narrateur|Une miette tombe près de la caisse.
-narrateur|Maman tient un filet de coton.
-narrateur|Le filet sent encore la lessive.
-narrateur|Le sol est un peu collant.
-maman|Tu as senti le pain, Nino ?
-enfant-m|Il est chaud.
-maman|Oui.
-maman|Il ira avec la tarte.
-narrateur|Nino touche le sac de pain.
-narrateur|Le papier est tiède.
-narrateur|En ce moment, Nino regarde les prunes.
-narrateur|Elles sont violettes et lisses.
-narrateur|Une caisse sent le sucré.
-enfant-m|J'en veux une ronde.
-enfant-m|Pour la tarte.
-maman|On en cherche une ferme.
-maman|Pas trop molle.
-narrateur|Mila arrive près de la caisse.
+          <t>narrateur|Une toile claque au-dessus des prunes.
+enfant-m|J'entends la toile, maman !
+maman|Tu l'entends, au-dessus ?
+enfant-m|Oui, elle claque.
+narrateur|Ça sent le sucré, un peu chaud.
+papa|Tu le sens, Nino ?
+enfant-m|Oui, papa.
+narrateur|Un cageot de bois est ouvert.
+narrateur|Des prunes violettes y brillent.
+narrateur|Sur la caisse, un éclat de cageot brille.
+enfant-m|Il brille, papa !
+papa|Tu le vois, sur le bois ?
+enfant-m|Oui, un petit point.
+maman|Le filet de coton est prêt.
+enfant-m|Il gratte un peu.
+maman|On le remplit, Nino ?
+enfant-m|Oui, avec une prune.
+narrateur|Le pain chaud tape le bras de Nino.
+enfant-m|Il est tiède.
+papa|Le papier croustille ?
+enfant-m|Oui, papa.
+narrateur|À côté, des pommes rouges attendent.
+enfant-m|Elles sont lisses, maman.
+maman|On verra les pommes après ?
+enfant-m|Après la prune.
+narrateur|Une balance fait tic, tout près.
+enfant-m|J'entends le tic.
+papa|C'est la balance ?
+enfant-m|Oui.
+narrateur|En ce moment, Nino veut une prune.
+enfant-m|Je veux une prune, maintenant !
+enfant-m|Une prune violette, maman.
+maman|Avec Mila, Nino ?
+enfant-m|Oui, maman.
+narrateur|Nino saisit trop vite une prune.
+narrateur|La prune glisse entre ses doigts.
+narrateur|Elle tombe dans le cageot.
+enfant-m|Elle est tombée !
+narrateur|Nino tire le filet trop vite.
+narrateur|Le filet se coince au bord.
+enfant-m|Il est coincé !
+papa|Le coton, Nino ?
+enfant-m|Il tient au bois.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu veux la prune avec Mila ?
+enfant-m|Oui, maman.
+papa|Tes mains sont collantes, Nino ?
+enfant-m|Un peu, papa.
+narrateur|Mila arrive près du cageot.
+enfant-m|Mila !
 narrateur|Ses chaussures collent un peu au sol.
 narrateur|Mila a des lunettes neuves.
-narrateur|Mila a les cheveux lisses.
+papa|Tu vois Mila, Nino ?
+enfant-m|Oui, papa.
+narrateur|Elles brillent un peu.
 narrateur|Elle porte un gilet vert.
-maman|Mila, tu cherches avec Nino.
-enfant-m|Tu m'aides, Mila ?
+enfant-m|Tu viens, Mila ?
 copine|Oui.
-narrateur|Nino prend une prune.
-narrateur|Elle cède un peu sous le doigt.
-enfant-m|Elle est molle.
-maman|On la repose.
-maman|Tout doux, dans la caisse.
-narrateur|Mila se penche sur la caisse.
-narrateur|Elle regarde au fond.
-copine|Au fond.
-copine|Celle-là.</t>
+narrateur|Nino ouvre la bouche.
+narrateur|Un petit rire commence.
+enfant-m|Oh.
+narrateur|Nino ferme la bouche.
+narrateur|Il regarde la caisse.
+narrateur|Il tend une prune.
+enfant-m|Pour toi.
+narrateur|Mila ne dit rien, d'abord.
+narrateur|Elle compte les prunes des yeux.
+copine|Celle-là.
+narrateur|L'éclat de cageot tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1397,22 +1436,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila a des lunettes. Que fait Nino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait Nino ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Inès a des lunettes. Que fait Maya ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait Nino ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jouer</t>
+          <t>pas rire</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | aider | prune | on joue | pas rire</t>
+          <t>pas rire | jouer | ensemble</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1427,7 +1466,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Nino écoute Mila. Que fait-il ?</t>
+          <t>On ne rit pas de l'apparence. Que fait Nino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1465,7 +1504,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1476,7 +1515,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1491,34 +1530,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,17 +1576,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_ferme_la_bouche_tend_la_prune; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1576,17 +1619,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino écoute Mila. Il prend la prune du fond. Elle est lisse et ferme. Merci, Nino. Merci, Mila. Elle est ronde. Pour la tarte. On la met dans le filet. Le filet s'alourdit un peu. Le coton se tend. Mila a vu au fond. On a la prune. On prend une pomme aussi ? Oui. Une pomme rouge. Mila montre une pomme brillante. Nino la pose dans le filet. Elle est lisse.</t>
+          <t>Nino veut une prune plus brillante. Celle-là brille plus ! Il avance trop vite vers la caisse. Les mots se bousculent dans sa bouche. Non. Mila recule d'un pas. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la main. Personne ne parle. Il observe le cageot, un instant. Nino regarde l'éclat de cageot. Tu veux la prune avec Mila ? Tu prends celle du fond ? Mila ne dit rien, d'abord. Elle pose le doigt sur une prune. Elle est ferme. D'accord. Nino la pose dans le filet. Le coton se tend un peu. Merci, Nino. Maman a vu la prune tendue. Mila, tu as vu le filet ? Oui. On prend une pomme aussi ? Une pomme rouge, Nino ? Oui, maman. Mila montre une pomme brillante. Nino la pose dans le filet. Elle est lisse. Le filet s'alourdit ? Un peu, papa. Tes mains sont propres, Nino ? Un peu collantes. Le ventre de Nino se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino écoute Mila. Il prend la prune du fond. Elle est lisse et ferme. Merci, Nino. Merci, Mila. Elle est ronde. Pour la tarte. On la met dans le filet. Le filet s'alourdit un peu. Le coton se tend. Mila a vu au fond. On a la prune. On prend une pomme aussi ? Oui. Une pomme rouge. Mila montre une pomme brillante. Nino la pose dans le filet. Elle est lisse.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut une prune plus brillante. Celle-là brille plus ! Il avance trop vite vers la caisse. Les mots se bousculent dans sa bouche. Non. Mila recule d'un pas. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la main. Personne ne parle. Il observe le cageot, un instant. Nino regarde l'éclat de cageot. Tu veux la prune avec Mila ? Tu prends celle du fond ? Mila ne dit rien, d'abord. Elle pose le doigt sur une prune. Elle est ferme. D'accord. Nino la pose dans le &lt;emphasis level="moderate"&gt;filet&lt;/emphasis&gt;. Le coton se tend un peu. Merci, Nino. Maman a vu la prune tendue. Mila, tu as vu le filet ? Oui. On prend une pomme aussi ? Une pomme rouge, Nino ? Oui, maman. Mila montre une pomme brillante. Nino la pose dans le filet. Elle est lisse. Le filet s'alourdit ? Un peu, papa. Tes mains sont propres, Nino ? Un peu collantes. Le ventre de Nino se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Maya n'a &lt;emphasis&gt;pas&lt;/emphasis&gt; ri. Elle a joué avec Inès. Pas rire de l'apparence. [pause]</t>
+          <t>Nino veut une prune plus brillante. Celle-là brille plus ! Il avance trop vite vers la caisse. Les mots se bousculent dans sa bouche. Non. Mila recule d'un pas. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la main. Personne ne parle. Il observe le cageot, un instant. Nino regarde l'éclat de cageot. Tu veux la prune avec Mila ? Tu prends celle du fond ? Mila ne dit rien, d'abord. Elle pose le doigt sur une prune. Elle est ferme. D'accord. Nino la pose dans le &lt;emphasis&gt;filet&lt;/emphasis&gt;. Le coton se tend un peu. Merci, Nino. Maman a vu la prune tendue. Mila, tu as vu le filet ? Oui. On prend une pomme aussi ? Une pomme rouge, Nino ? Oui, maman. Mila montre une pomme brillante. Nino la pose dans le filet. Elle est lisse. Le filet s'alourdit ? Un peu, papa. Tes mains sont propres, Nino ? Un peu collantes. Le ventre de Nino se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,7 +1676,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1641,10 +1684,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,30 +1710,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>filet</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1699,10 +1742,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1715,29 +1758,52 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_ils_posent_la_prune; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino écoute Mila.
-narrateur|Il prend la prune du fond.
-narrateur|Elle est lisse et ferme.
+          <t>narrateur|Nino veut une prune plus brillante.
+enfant-m|Celle-là brille plus !
+narrateur|Il avance trop vite vers la caisse.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Mila recule d'un pas.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nino refuse de foncer.
+narrateur|Il referme la main.
+narrateur|Personne ne parle.
+narrateur|Il observe le cageot, un instant.
+narrateur|Nino regarde l'éclat de cageot.
+papa|Tu veux la prune avec Mila ?
+enfant-m|Tu prends celle du fond ?
+narrateur|Mila ne dit rien, d'abord.
+narrateur|Elle pose le doigt sur une prune.
+copine|Elle est ferme.
+enfant-m|D'accord.
+narrateur|Nino la pose dans le filet.
+narrateur|Le coton se tend un peu.
 maman|Merci, Nino.
-maman|Merci, Mila.
-enfant-m|Elle est ronde.
-copine|Pour la tarte.
-maman|On la met dans le filet.
-narrateur|Le filet s'alourdit un peu.
-narrateur|Le coton se tend.
-maman|Mila a vu au fond.
-maman|On a la prune.
+narrateur|Maman a vu la prune tendue.
+papa|Mila, tu as vu le filet ?
+copine|Oui.
 enfant-m|On prend une pomme aussi ?
-maman|Oui.
-maman|Une pomme rouge.
+maman|Une pomme rouge, Nino ?
+enfant-m|Oui, maman.
 narrateur|Mila montre une pomme brillante.
 narrateur|Nino la pose dans le filet.
-enfant-m|Elle est lisse.</t>
+enfant-m|Elle est lisse.
+papa|Le filet s'alourdit ?
+enfant-m|Un peu, papa.
+maman|Tes mains sont propres, Nino ?
+enfant-m|Un peu collantes.
+narrateur|Le ventre de Nino se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>filet,prune</t>
         </is>
       </c>
     </row>
@@ -1764,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>La pomme rejoint la prune. Le filet balance. Il est lourd, le filet ? Un peu. On le porte à deux. Nino tient une anse. Maman tient l'autre. Mila marche tout près. Un stand de menthe sent fort. Ça pique le nez. C'est la menthe. C'est vert. Vert et frais. Ils passent près des œufs. Les boîtes sont beiges. Bravo. Tu as choisi la prune ferme. Le pain chaud tape le bras. Ce soir, la tarte. Oui. Avec ta prune ronde. Et la pomme. Une balance fait tic près d'eux. Les toiles claquent un peu.</t>
+          <t>Nino veut montrer la prune brillante. Je la porte, maintenant ! Il lève le filet trop haut. Attends. Trop vite, d'un coup. Une prune presse contre le coton. Ça tache ! Un peu de jus glisse sur le gilet. Le gilet, Nino ? Il est taché. Les lunettes de Mila bougent. Nino ouvre la bouche. Un petit rire revient, presque. Oh. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite à voix haute. Il observe le filet, un instant. Il écoute le tic de la balance. Sur la caisse, un éclat de cageot luit. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Le filet, Nino ? On le porte à deux. Nino tient une anse. Mila tient l'autre. Je le tiens. Ils marchent, sans se presser. C'est passé. Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>La pomme rejoint la prune. Le filet balance. Il est lourd, le filet ? Un peu. On le porte à deux. Nino tient une anse. Maman tient l'autre. Mila marche tout près. Un stand de menthe sent fort. Ça pique le nez. C'est la menthe. C'est vert. Vert et frais. Ils passent près des œufs. Les boîtes sont beiges. Bravo. Tu as choisi la prune ferme. Le pain chaud tape le bras. Ce soir, la tarte. Oui. Avec ta prune ronde. Et la pomme. Une balance fait tic près d'eux. Les toiles claquent un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nino veut montrer la prune brillante. Je la porte, maintenant ! Il lève le filet trop haut. Attends. Trop vite, d'un coup. Une prune presse contre le coton. Ça tache ! Un peu de jus glisse sur le gilet. Le gilet, Nino ? Il est taché. Les lunettes de Mila bougent. Nino ouvre la bouche. Un petit rire revient, presque. Oh. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite à voix haute. Il observe le filet, un instant. Il écoute le tic de la balance. Sur la caisse, un &lt;emphasis level="moderate"&gt;éclat de cageot&lt;/emphasis&gt; luit. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Le filet, Nino ? On le porte à deux. Nino tient une anse. Mila tient l'autre. Je le tiens. Ils marchent, sans se presser. C'est passé. Oui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman achète du pain. Maya donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Nino veut montrer la prune brillante. Je la porte, maintenant ! Il lève le filet trop haut. Attends. Trop vite, d'un coup. Une prune presse contre le coton. Ça tache ! Un peu de jus glisse sur le gilet. Le gilet, Nino ? Il est taché. Les lunettes de Mila bougent. Nino ouvre la bouche. Un petit rire revient, presque. Oh. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite à voix haute. Il observe le filet, un instant. Il écoute le tic de la balance. Sur la caisse, un &lt;emphasis&gt;éclat de cageot&lt;/emphasis&gt; luit. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Le filet, Nino ? On le porte à deux. Nino tient une anse. Mila tient l'autre. Je le tiens. Ils marchent, sans se presser. C'est passé. Oui.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1821,7 +1887,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1829,22 +1895,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1855,30 +1925,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de cageot</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,47 +1957,63 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|La pomme rejoint la prune.
-narrateur|Le filet balance.
-maman|Il est lourd, le filet ?
-enfant-m|Un peu.
-maman|On le porte à deux.
+          <t>narrateur|Nino veut montrer la prune brillante.
+enfant-m|Je la porte, maintenant !
+narrateur|Il lève le filet trop haut.
+copine|Attends.
+narrateur|Trop vite, d'un coup.
+narrateur|Une prune presse contre le coton.
+enfant-m|Ça tache !
+narrateur|Un peu de jus glisse sur le gilet.
+papa|Le gilet, Nino ?
+enfant-m|Il est taché.
+narrateur|Les lunettes de Mila bougent.
+narrateur|Nino ouvre la bouche.
+narrateur|Un petit rire revient, presque.
+enfant-m|Oh.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Il observe le filet, un instant.
+narrateur|Il écoute le tic de la balance.
+narrateur|Sur la caisse, un éclat de cageot luit.
+enfant-m|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bois.
+maman|Le filet, Nino ?
+enfant-m|On le porte à deux.
 narrateur|Nino tient une anse.
-narrateur|Maman tient l'autre.
-narrateur|Mila marche tout près.
-narrateur|Un stand de menthe sent fort.
-enfant-m|Ça pique le nez.
-maman|C'est la menthe.
-copine|C'est vert.
-maman|Vert et frais.
-narrateur|Ils passent près des œufs.
-narrateur|Les boîtes sont beiges.
-maman|Bravo.
-maman|Tu as choisi la prune ferme.
-narrateur|Le pain chaud tape le bras.
-enfant-m|Ce soir, la tarte.
-maman|Oui.
-maman|Avec ta prune ronde.
-copine|Et la pomme.
-narrateur|Une balance fait tic près d'eux.
-narrateur|Les toiles claquent un peu.</t>
+narrateur|Mila tient l'autre.
+copine|Je le tiens.
+narrateur|Ils marchent, sans se presser.
+enfant-m|C'est passé.
+copine|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>marche,filet</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2040,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient la prune et la pomme. Le sac de pain sent le four. On a la prune de la tarte. Oui. Vous avez cherché ensemble. La farine reste sur la planche.</t>
+          <t>Un stand de menthe sent fort. Ça pique le nez, maman. C'est la menthe ? Oui, vert et frais. Tu la sens, Nino ? Oui, papa. Ils passent près des œufs. Les boîtes sont beiges. Tu vois les boîtes, Nino ? Oui, papa. Ils s'assoient sur le banc. On est bien, ici. On a la prune, papa. Tu la vois, dans le filet ? Oui, avec Mila. Et la pomme. Nino pose la prune entre eux. Mila pose la main près. Elle est à nous. Elle est là, Nino. Oui, maman. Le pain chaud reste contre le bras. L'éclat est là, papa. Tu le vois sur le bois ? Oui, papa. Les toiles claquent un peu. Un éclat de cageot tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient la prune et la pomme. Le sac de pain sent le four. On a la prune de la tarte. Oui. Vous avez cherché ensemble. La farine reste sur la planche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un stand de menthe sent fort. Ça pique le nez, maman. C'est la menthe ? Oui, vert et frais. Tu la sens, Nino ? Oui, papa. Ils passent près des œufs. Les boîtes sont beiges. Tu vois les boîtes, Nino ? Oui, papa. Ils s'assoient sur le banc. On est bien, ici. On a la prune, papa. Tu la vois, dans le filet ? Oui, avec Mila. Et la pomme. Nino pose la prune entre eux. Mila pose la main près. Elle est à nous. Elle est là, Nino. Oui, maman. Le pain chaud reste contre le bras. L'éclat est là, papa. Tu le vois sur le bois ? Oui, papa. Les toiles claquent un peu. Un &lt;emphasis level="moderate"&gt;éclat de cageot&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un stand de menthe sent fort. Ça pique le nez, maman. C'est la menthe ? Oui, vert et frais. Tu la sens, Nino ? Oui, papa. Ils passent près des œufs. Les boîtes sont beiges. Tu vois les boîtes, Nino ? Oui, papa. Ils s'assoient sur le banc. On est bien, ici. On a la prune, papa. Tu la vois, dans le filet ? Oui, avec Mila. Et la pomme. Nino pose la prune entre eux. Mila pose la main près. Elle est à nous. Elle est là, Nino. Oui, maman. Le pain chaud reste contre le bras. L'éclat est là, papa. Tu le vois sur le bois ? Oui, papa. Les toiles claquent un peu. Un &lt;emphasis&gt;éclat de cageot&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2097,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2117,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2131,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cageot</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2154,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,29 +2167,59 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le filet tient la prune et la pomme.
-narrateur|Le sac de pain sent le four.
-enfant-m|On a la prune de la tarte.
-maman|Oui.
-maman|Vous avez cherché ensemble.
-narrateur|La farine reste sur la planche.</t>
+          <t>narrateur|Un stand de menthe sent fort.
+enfant-m|Ça pique le nez, maman.
+maman|C'est la menthe ?
+enfant-m|Oui, vert et frais.
+papa|Tu la sens, Nino ?
+enfant-m|Oui, papa.
+narrateur|Ils passent près des œufs.
+narrateur|Les boîtes sont beiges.
+papa|Tu vois les boîtes, Nino ?
+enfant-m|Oui, papa.
+narrateur|Ils s'assoient sur le banc.
+maman|On est bien, ici.
+enfant-m|On a la prune, papa.
+papa|Tu la vois, dans le filet ?
+enfant-m|Oui, avec Mila.
+copine|Et la pomme.
+narrateur|Nino pose la prune entre eux.
+narrateur|Mila pose la main près.
+enfant-m|Elle est à nous.
+maman|Elle est là, Nino.
+enfant-m|Oui, maman.
+narrateur|Le pain chaud reste contre le bras.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur le bois ?
+enfant-m|Oui, papa.
+narrateur|Les toiles claquent un peu.
+narrateur|Un éclat de cageot tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>prune,menthe</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2205,6 +2325,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>